<commit_message>
Update 1 số function
Update 1 số function
</commit_message>
<xml_diff>
--- a/SmartBooks.HumanResource/bin/x86/Debug/Teamleate/DanhSachNhanVienMoiVao.xlsx
+++ b/SmartBooks.HumanResource/bin/x86/Debug/Teamleate/DanhSachNhanVienMoiVao.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SourceCodeHR\SnK_Dev\SmartBooks.HumanResource\bin\x86\Debug\Teamleate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C8E985-1DEB-4352-8632-9BD5959FDAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A923DB-1B78-45B5-846A-35706E05E863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>